<commit_message>
Se añade la generación de Javadocs
Se corrigen comentarios incorrectos.
Se añade a Security el directorio de javadocs

Se retoca "miperfil" y cambio de password.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/docs/Casos de uso.xlsx
+++ b/src/main/resources/static/docs/Casos de uso.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\prueba\uned-aplicacionweb\src\main\resources\static\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E12B5AD-682F-491C-8922-522DE20D43B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1035BF87-C39E-42D7-AB51-13ED18C917C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D444AEC3-67F7-4F7F-BD45-FBD327D01921}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{D444AEC3-67F7-4F7F-BD45-FBD327D01921}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="CU-001" sheetId="1" r:id="rId1"/>
+    <sheet name="CU-001 (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,10 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>CASO DE USO</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
   <si>
     <t>Actores</t>
   </si>
@@ -64,6 +62,51 @@
   </si>
   <si>
     <t>Cursos alternativos</t>
+  </si>
+  <si>
+    <t>Usuario anónimo</t>
+  </si>
+  <si>
+    <t>Gestión de cursos, Gestión de Áreas</t>
+  </si>
+  <si>
+    <t>El usuario accede a la plataforma y revisar los cursos existentees.</t>
+  </si>
+  <si>
+    <t>Búsqueda de cursos</t>
+  </si>
+  <si>
+    <t>El usuario navega por los cursos y puede visualizar el contenido ndividual de cada uno.</t>
+  </si>
+  <si>
+    <t>CU-001 - Consulta de Cursos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.-El usuario navega (con las flechas de desplazamiento) por los diferentes cursos. </t>
+  </si>
+  <si>
+    <t>2.- El usuario selecciona (pulsando sobre la opción de "Ver Curso"), el curso deseado.</t>
+  </si>
+  <si>
+    <t>Primario</t>
+  </si>
+  <si>
+    <t>CU-002 - Búsqueda por Areas de interes</t>
+  </si>
+  <si>
+    <t>Se obtiene la visualización de los cursos del área seleccionada.</t>
+  </si>
+  <si>
+    <t>El usuario accede a la plataforma y selecciona un Área de interes.</t>
+  </si>
+  <si>
+    <t>1.-El usuario selecciona un área de interés y pulsa sobre el icono "Buscar"</t>
+  </si>
+  <si>
+    <t>2.- Se filtran los cursos de esa área y se muestran los resultados de las 3 categorías.</t>
+  </si>
+  <si>
+    <t>Si no existen cursos, se visualizará un aviso "No hay cursos disponibles en este momento".</t>
   </si>
 </sst>
 </file>
@@ -216,32 +259,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -250,11 +293,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -579,67 +634,189 @@
   <sheetData>
     <row r="2" spans="3:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="3:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+    </row>
+    <row r="4" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="2"/>
+      <c r="D4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="10"/>
+    </row>
+    <row r="5" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="12"/>
+    </row>
+    <row r="6" spans="3:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="15"/>
+    </row>
+    <row r="7" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="12"/>
+    </row>
+    <row r="8" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="12"/>
+    </row>
+    <row r="9" spans="3:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="C9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="18"/>
+    </row>
+    <row r="10" spans="3:5" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="5"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0254D140-2508-4104-9B8E-E530EA4DAADA}">
+  <dimension ref="C2:E11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="4" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="38.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="3:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="10"/>
+    </row>
+    <row r="5" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="14"/>
-    </row>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="12"/>
+    </row>
+    <row r="6" spans="3:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="12"/>
-    </row>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="15"/>
+    </row>
+    <row r="7" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="12"/>
+    </row>
+    <row r="8" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="12"/>
+    </row>
+    <row r="9" spans="3:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="C9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="12"/>
-    </row>
-    <row r="9" spans="3:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="18"/>
+    </row>
+    <row r="10" spans="3:5" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="8"/>
-    </row>
-    <row r="10" spans="3:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="C11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="10"/>
-    </row>
-    <row r="11" spans="3:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="C11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="8"/>
+      <c r="D11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
documentos para la memoria
</commit_message>
<xml_diff>
--- a/src/main/resources/static/docs/Casos de uso.xlsx
+++ b/src/main/resources/static/docs/Casos de uso.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\prueba\uned-aplicacionweb\src\main\resources\static\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1035BF87-C39E-42D7-AB51-13ED18C917C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C46BB7-7B62-452B-9391-034E29E3ADE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{D444AEC3-67F7-4F7F-BD45-FBD327D01921}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{D444AEC3-67F7-4F7F-BD45-FBD327D01921}"/>
   </bookViews>
   <sheets>
     <sheet name="CU-001" sheetId="1" r:id="rId1"/>
-    <sheet name="CU-001 (2)" sheetId="2" r:id="rId2"/>
+    <sheet name="CU-002" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -85,9 +85,6 @@
     <t xml:space="preserve">1.-El usuario navega (con las flechas de desplazamiento) por los diferentes cursos. </t>
   </si>
   <si>
-    <t>2.- El usuario selecciona (pulsando sobre la opción de "Ver Curso"), el curso deseado.</t>
-  </si>
-  <si>
     <t>Primario</t>
   </si>
   <si>
@@ -107,6 +104,9 @@
   </si>
   <si>
     <t>Si no existen cursos, se visualizará un aviso "No hay cursos disponibles en este momento".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.- Se ejecutan las consultas de los cursos de las 3 categorías y se muestra en formato "carrusel" de fichas (3 por categoría). </t>
   </si>
 </sst>
 </file>
@@ -672,7 +672,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" s="12"/>
     </row>
@@ -702,7 +702,7 @@
         <v>14</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="3:5" ht="30" x14ac:dyDescent="0.25">
@@ -739,7 +739,7 @@
     <row r="2" spans="3:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="3:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C3" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="8"/>
@@ -767,7 +767,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" s="15"/>
     </row>
@@ -776,7 +776,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" s="12"/>
     </row>
@@ -785,7 +785,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E8" s="12"/>
     </row>
@@ -803,10 +803,10 @@
         <v>6</v>
       </c>
       <c r="D10" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="16" t="s">
         <v>20</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="11" spans="3:5" ht="30" x14ac:dyDescent="0.25">
@@ -814,7 +814,7 @@
         <v>7</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E11" s="5"/>
     </row>

</xml_diff>